<commit_message>
Dashboard base code finalised, I removed old commented code which is not being used, debugged the code entirely. Fixed up presentation and condensed some unecessary extra bits in the code to be shorter more effective and presentable.
</commit_message>
<xml_diff>
--- a/Brief and files/heart failure data catalogue With Data.xlsx
+++ b/Brief and files/heart failure data catalogue With Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noahaslan/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noahaslan/Desktop/Uni Work/Oxford Brookes/Year 3 Uni work/COMP 6013 Project:Dissertation/Dashboard code folder/Brief and files/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C6B9646-7265-E144-AFBB-8155B1D1E6D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17120" activeTab="1" xr2:uid="{BCC61590-1505-46FA-AFC9-CAD58C82448A}"/>
+    <workbookView xWindow="20" yWindow="660" windowWidth="30240" windowHeight="17120" activeTab="1" xr2:uid="{BCC61590-1505-46FA-AFC9-CAD58C82448A}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover sheet" sheetId="3" r:id="rId1"/>
@@ -4037,6 +4037,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_activity xmlns="d4138443-ee6d-4b26-8b57-d94a58805224" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100148D45EC9781F949A0CAA7115F2F2010" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5eb2a6caf9d93b40a01c0cf8a8efce3f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns3="d4138443-ee6d-4b26-8b57-d94a58805224" xmlns:ns4="8474001e-63e9-4a93-9c01-a8f0bfa29f8b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff2e2e1b8afe4b7b2d66968e54e0e9c4" ns1:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -4280,26 +4299,33 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CC53B54-5460-44CF-969B-84BEA4BC1063}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="8474001e-63e9-4a93-9c01-a8f0bfa29f8b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d4138443-ee6d-4b26-8b57-d94a58805224"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_activity xmlns="d4138443-ee6d-4b26-8b57-d94a58805224" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{180FD8C1-991A-498A-9357-2A5B0C5ECE67}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32FF6341-1B81-42DC-B813-655E42F9B03A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4317,30 +4343,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{180FD8C1-991A-498A-9357-2A5B0C5ECE67}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CC53B54-5460-44CF-969B-84BEA4BC1063}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="8474001e-63e9-4a93-9c01-a8f0bfa29f8b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d4138443-ee6d-4b26-8b57-d94a58805224"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>